<commit_message>
Add solutions for LC 1359, 187, 936, 2472 and update trackers
Solutions:
- 1359: Count All Valid Pickup and Delivery Options (Math/Combinatorics)
- 187: Repeated DNA Sequences (String/Rolling Hash)
- 936: Stamping the Sequence (Greedy/Reverse Simulation)
- 2472: Maximum Number of Non-Overlapping Palindrome Substrings (Palindrome DP)
- math/hull: CHT/duality diagram (scratch notes)

Tracker updates:
- Global_tracker.XLSX: added rows for all 4 problems
- google_prep_questions.xlsx: added rows for all 4 problems
- google_prep_tracker.md: removed solved entries, renumbered sections,
  bumped Hard Problems Goal to 151/200 (76%)
- string/patterns.md: rolling hash gotchas

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Progress/Company wise/google/google_prep_questions.xlsx
+++ b/Progress/Company wise/google/google_prep_questions.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3706,7 +3706,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>1.8 DP - Advanced</t>
+          <t>1.9 Maths</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3732,6 +3732,134 @@
       <c r="G92" t="inlineStr">
         <is>
           <t>Array / Math / Number Theory / GCD</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1.9 Maths</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Count All Valid Pickup and Delivery Options</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>1359</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Math / Combinatorics / AP Series</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1.11 String - Advanced</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Repeated DNA Sequences</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>String / Rolling Hash / Rabin-Karp</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1.10 Greedy</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Stamping the Sequence</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>936</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>String / Greedy / Reverse Simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1.11 String - Advanced</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Maximum Number of Non-Overlapping Palindrome Substrings</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2472</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>String / Palindrome DP / Interval DP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add solutions for LC 1510, 464 and update trackers + patterns
Solutions:
- 1510: Stone Game IV (Game Theory/Sprague-Grundy/DP)
- 464: Can I Win (Game Theory/Bitmask DP/Memoized Search)

Patterns:
- game theory/patterns.md: new Bitmask DP / Memoized Game State Search
  section distinguishing it from Sprague-Grundy; documents 3 bugs found
  in LC 464 (redundant memo key -> MLE, broken OR-based cache check,
  missing target-unreachable guard)
- dp/patterns.md: generalized the same 2 gotchas (derivable memo keys
  causing MLE, minimal-exact memo keys, reachability guards) to
  bitmask DP and memoized recursion broadly

Tracker updates:
- Global_tracker.XLSX: added rows for both problems
- google_prep_questions.xlsx: added rows for both problems
- google_prep_tracker.md: removed solved entries, renumbered sections,
  bumped Hard Problems Goal to 152/200 (77%) for LC 1510 (LC 464 is
  Medium, counter untouched)

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Progress/Company wise/google/google_prep_questions.xlsx
+++ b/Progress/Company wise/google/google_prep_questions.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3863,6 +3863,70 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1.12 Game Theory</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Stone Game IV</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Game Theory / Sprague-Grundy / DP</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1.12 Game Theory</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Can I Win</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>464</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Game Theory / Bitmask DP / Memoized Search</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>